<commit_message>
适配mac/低内存 	modified:   0 zombie type/quick/main_quick_show.cpp 	new file:   "0 zombie type/\351\230\263\345\205\211\346\250\241\345\236\213/12-1 NE 1.5\350\212\261\344\272\224\345\205\253 hqyx/3\351\230\263\345\205\211\344\274\260\350\256\241-\347\240\264\351\230\265\347\216\207slow.cpp" 	modified:   "0 zombie type/\351\230\263\345\205\211\346\250\241\345\236\213/12-1 NE 1.5\350\212\261\344\272\224\345\205\253 hqyx/3\351\230\263\345\205\211\346\200\273\347\273\223.xlsx" 	modified:   inc/basic_setting.h
</commit_message>
<xml_diff>
--- a/0 zombie type/阳光模型/12-1 NE 1.5花五八 hqyx/3阳光总结.xlsx
+++ b/0 zombie type/阳光模型/12-1 NE 1.5花五八 hqyx/3阳光总结.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="7380" windowHeight="12300"/>
+    <workbookView windowHeight="15100"/>
   </bookViews>
   <sheets>
     <sheet name="破阵率" sheetId="2" r:id="rId1"/>
@@ -1038,7 +1038,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B1:D4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="3" outlineLevelCol="3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="3" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="3" width="9" style="1"/>
     <col min="4" max="4" width="9.375" style="1"/>
@@ -1068,18 +1068,22 @@
         <v>3</v>
       </c>
       <c r="C3" s="4">
-        <v>0</v>
+        <v>17.1</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2">
+        <v>15</v>
+      </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="4">
-        <v>0</v>
+        <v>95.42</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2">
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>